<commit_message>
Cap nhat du lieu - 07/05/2026 14:57
</commit_message>
<xml_diff>
--- a/PM_092.xlsx
+++ b/PM_092.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1. TCKT_PCVT\2.SCL\2026\Báo cáo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TUAN HOC A.I\1. TCKT_PCVT\4. Công nghệ AI\KT SCL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{298DDB8B-3D55-4527-A226-2A59937B3999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{937510B4-8285-42FF-8E17-8B3A854FDBE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{AC1AAD16-9061-42F9-B216-D7E5AB78D483}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1061" uniqueCount="144">
   <si>
     <t>TỔNG CÔNG TY ĐIỆN LỰC THÀNH PHỐ HỒ CHÍ MINH TNHH</t>
   </si>
@@ -1769,10 +1769,6 @@
     <xf numFmtId="0" fontId="25" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
@@ -1782,8 +1778,11 @@
     <xf numFmtId="0" fontId="21" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1793,12 +1792,6 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1812,6 +1805,13 @@
     <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2187,7 +2187,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC097D15-D4E4-46F1-B3C8-4A7361019462}">
-  <dimension ref="A1:H265"/>
+  <dimension ref="A1:H267"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.19921875" bestFit="1" customWidth="1"/>
@@ -2249,98 +2249,98 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="35"/>
+      <c r="H12" s="35"/>
     </row>
     <row r="13" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="C13" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="D13" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="E13" s="34" t="s">
+      <c r="E13" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="F13" s="35"/>
-      <c r="G13" s="30" t="s">
+      <c r="F13" s="32"/>
+      <c r="G13" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="30" t="s">
+      <c r="H13" s="24" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="33"/>
-      <c r="B14" s="33"/>
-      <c r="C14" s="33"/>
-      <c r="D14" s="33"/>
+      <c r="A14" s="30"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="25"/>
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="29"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="28"/>
     </row>
     <row r="16" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="29"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="28"/>
     </row>
     <row r="17" spans="1:8" ht="18.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="29"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="28"/>
     </row>
     <row r="18" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="23" t="s">
+      <c r="A18" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="25"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="23"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
@@ -2899,12 +2899,12 @@
       </c>
     </row>
     <row r="42" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="23" t="s">
+      <c r="A42" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B42" s="24"/>
-      <c r="C42" s="24"/>
-      <c r="D42" s="25"/>
+      <c r="B42" s="22"/>
+      <c r="C42" s="22"/>
+      <c r="D42" s="23"/>
       <c r="E42" s="13">
         <v>103128028</v>
       </c>
@@ -2913,12 +2913,12 @@
       <c r="H42" s="7"/>
     </row>
     <row r="43" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="23" t="s">
+      <c r="A43" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B43" s="24"/>
-      <c r="C43" s="24"/>
-      <c r="D43" s="25"/>
+      <c r="B43" s="22"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="23"/>
       <c r="E43" s="13">
         <v>103128028</v>
       </c>
@@ -2927,24 +2927,24 @@
       <c r="H43" s="7"/>
     </row>
     <row r="44" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="23" t="s">
+      <c r="A44" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B44" s="24"/>
-      <c r="C44" s="24"/>
-      <c r="D44" s="25"/>
+      <c r="B44" s="22"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="23"/>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
       <c r="H44" s="7"/>
     </row>
     <row r="45" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="23" t="s">
+      <c r="A45" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="B45" s="24"/>
-      <c r="C45" s="24"/>
-      <c r="D45" s="25"/>
+      <c r="B45" s="22"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="23"/>
       <c r="E45" s="13">
         <v>103128028</v>
       </c>
@@ -2953,12 +2953,12 @@
       <c r="H45" s="7"/>
     </row>
     <row r="46" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="23" t="s">
+      <c r="A46" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B46" s="24"/>
-      <c r="C46" s="24"/>
-      <c r="D46" s="25"/>
+      <c r="B46" s="22"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="23"/>
       <c r="E46" s="13">
         <v>103128028</v>
       </c>
@@ -2967,24 +2967,24 @@
       <c r="H46" s="7"/>
     </row>
     <row r="47" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="23" t="s">
+      <c r="A47" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B47" s="24"/>
-      <c r="C47" s="24"/>
-      <c r="D47" s="25"/>
+      <c r="B47" s="22"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="23"/>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
       <c r="G47" s="7"/>
       <c r="H47" s="7"/>
     </row>
     <row r="48" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="23" t="s">
+      <c r="A48" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="B48" s="24"/>
-      <c r="C48" s="24"/>
-      <c r="D48" s="25"/>
+      <c r="B48" s="22"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="23"/>
       <c r="E48" s="13">
         <v>103128028</v>
       </c>
@@ -2993,12 +2993,12 @@
       <c r="H48" s="7"/>
     </row>
     <row r="49" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="23" t="s">
+      <c r="A49" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B49" s="24"/>
-      <c r="C49" s="24"/>
-      <c r="D49" s="25"/>
+      <c r="B49" s="22"/>
+      <c r="C49" s="22"/>
+      <c r="D49" s="23"/>
       <c r="E49" s="13">
         <v>103128028</v>
       </c>
@@ -3007,48 +3007,48 @@
       <c r="H49" s="7"/>
     </row>
     <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="27" t="s">
+      <c r="A50" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B50" s="28"/>
-      <c r="C50" s="28"/>
-      <c r="D50" s="28"/>
-      <c r="E50" s="28"/>
-      <c r="F50" s="28"/>
-      <c r="G50" s="28"/>
-      <c r="H50" s="29"/>
+      <c r="B50" s="27"/>
+      <c r="C50" s="27"/>
+      <c r="D50" s="27"/>
+      <c r="E50" s="27"/>
+      <c r="F50" s="27"/>
+      <c r="G50" s="27"/>
+      <c r="H50" s="28"/>
     </row>
     <row r="51" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="27" t="s">
+      <c r="A51" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B51" s="28"/>
-      <c r="C51" s="28"/>
-      <c r="D51" s="28"/>
-      <c r="E51" s="28"/>
-      <c r="F51" s="28"/>
-      <c r="G51" s="28"/>
-      <c r="H51" s="29"/>
+      <c r="B51" s="27"/>
+      <c r="C51" s="27"/>
+      <c r="D51" s="27"/>
+      <c r="E51" s="27"/>
+      <c r="F51" s="27"/>
+      <c r="G51" s="27"/>
+      <c r="H51" s="28"/>
     </row>
     <row r="52" spans="1:8" ht="18.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="27" t="s">
+      <c r="A52" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B52" s="28"/>
-      <c r="C52" s="28"/>
-      <c r="D52" s="28"/>
-      <c r="E52" s="28"/>
-      <c r="F52" s="28"/>
-      <c r="G52" s="28"/>
-      <c r="H52" s="29"/>
+      <c r="B52" s="27"/>
+      <c r="C52" s="27"/>
+      <c r="D52" s="27"/>
+      <c r="E52" s="27"/>
+      <c r="F52" s="27"/>
+      <c r="G52" s="27"/>
+      <c r="H52" s="28"/>
     </row>
     <row r="53" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="23" t="s">
+      <c r="A53" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="B53" s="24"/>
-      <c r="C53" s="24"/>
-      <c r="D53" s="25"/>
+      <c r="B53" s="22"/>
+      <c r="C53" s="22"/>
+      <c r="D53" s="23"/>
       <c r="E53" s="7"/>
       <c r="F53" s="7"/>
       <c r="G53" s="7"/>
@@ -6775,12 +6775,12 @@
       </c>
     </row>
     <row r="209" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A209" s="23" t="s">
+      <c r="A209" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B209" s="24"/>
-      <c r="C209" s="24"/>
-      <c r="D209" s="25"/>
+      <c r="B209" s="22"/>
+      <c r="C209" s="22"/>
+      <c r="D209" s="23"/>
       <c r="E209" s="13">
         <v>1475408160</v>
       </c>
@@ -6791,12 +6791,12 @@
       <c r="H209" s="7"/>
     </row>
     <row r="210" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A210" s="23" t="s">
+      <c r="A210" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B210" s="24"/>
-      <c r="C210" s="24"/>
-      <c r="D210" s="25"/>
+      <c r="B210" s="22"/>
+      <c r="C210" s="22"/>
+      <c r="D210" s="23"/>
       <c r="E210" s="13">
         <v>1445729378</v>
       </c>
@@ -6805,24 +6805,24 @@
       <c r="H210" s="7"/>
     </row>
     <row r="211" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A211" s="23" t="s">
+      <c r="A211" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B211" s="24"/>
-      <c r="C211" s="24"/>
-      <c r="D211" s="25"/>
+      <c r="B211" s="22"/>
+      <c r="C211" s="22"/>
+      <c r="D211" s="23"/>
       <c r="E211" s="7"/>
       <c r="F211" s="7"/>
       <c r="G211" s="7"/>
       <c r="H211" s="7"/>
     </row>
     <row r="212" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A212" s="23" t="s">
+      <c r="A212" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="B212" s="24"/>
-      <c r="C212" s="24"/>
-      <c r="D212" s="25"/>
+      <c r="B212" s="22"/>
+      <c r="C212" s="22"/>
+      <c r="D212" s="23"/>
       <c r="E212" s="13">
         <v>1475408160</v>
       </c>
@@ -6833,12 +6833,12 @@
       <c r="H212" s="7"/>
     </row>
     <row r="213" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A213" s="23" t="s">
+      <c r="A213" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B213" s="24"/>
-      <c r="C213" s="24"/>
-      <c r="D213" s="25"/>
+      <c r="B213" s="22"/>
+      <c r="C213" s="22"/>
+      <c r="D213" s="23"/>
       <c r="E213" s="13">
         <v>1445729378</v>
       </c>
@@ -6847,24 +6847,24 @@
       <c r="H213" s="7"/>
     </row>
     <row r="214" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A214" s="23" t="s">
+      <c r="A214" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B214" s="24"/>
-      <c r="C214" s="24"/>
-      <c r="D214" s="25"/>
+      <c r="B214" s="22"/>
+      <c r="C214" s="22"/>
+      <c r="D214" s="23"/>
       <c r="E214" s="7"/>
       <c r="F214" s="7"/>
       <c r="G214" s="7"/>
       <c r="H214" s="7"/>
     </row>
     <row r="215" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A215" s="23" t="s">
+      <c r="A215" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="B215" s="24"/>
-      <c r="C215" s="24"/>
-      <c r="D215" s="25"/>
+      <c r="B215" s="22"/>
+      <c r="C215" s="22"/>
+      <c r="D215" s="23"/>
       <c r="E215" s="13">
         <v>1475408160</v>
       </c>
@@ -6875,12 +6875,12 @@
       <c r="H215" s="7"/>
     </row>
     <row r="216" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A216" s="23" t="s">
+      <c r="A216" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B216" s="24"/>
-      <c r="C216" s="24"/>
-      <c r="D216" s="25"/>
+      <c r="B216" s="22"/>
+      <c r="C216" s="22"/>
+      <c r="D216" s="23"/>
       <c r="E216" s="13">
         <v>1445729378</v>
       </c>
@@ -6889,48 +6889,48 @@
       <c r="H216" s="7"/>
     </row>
     <row r="217" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A217" s="27" t="s">
+      <c r="A217" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="B217" s="28"/>
-      <c r="C217" s="28"/>
-      <c r="D217" s="28"/>
-      <c r="E217" s="28"/>
-      <c r="F217" s="28"/>
-      <c r="G217" s="28"/>
-      <c r="H217" s="29"/>
+      <c r="B217" s="27"/>
+      <c r="C217" s="27"/>
+      <c r="D217" s="27"/>
+      <c r="E217" s="27"/>
+      <c r="F217" s="27"/>
+      <c r="G217" s="27"/>
+      <c r="H217" s="28"/>
     </row>
     <row r="218" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A218" s="27" t="s">
+      <c r="A218" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="B218" s="28"/>
-      <c r="C218" s="28"/>
-      <c r="D218" s="28"/>
-      <c r="E218" s="28"/>
-      <c r="F218" s="28"/>
-      <c r="G218" s="28"/>
-      <c r="H218" s="29"/>
+      <c r="B218" s="27"/>
+      <c r="C218" s="27"/>
+      <c r="D218" s="27"/>
+      <c r="E218" s="27"/>
+      <c r="F218" s="27"/>
+      <c r="G218" s="27"/>
+      <c r="H218" s="28"/>
     </row>
     <row r="219" spans="1:8" ht="18.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A219" s="27" t="s">
+      <c r="A219" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B219" s="28"/>
-      <c r="C219" s="28"/>
-      <c r="D219" s="28"/>
-      <c r="E219" s="28"/>
-      <c r="F219" s="28"/>
-      <c r="G219" s="28"/>
-      <c r="H219" s="29"/>
+      <c r="B219" s="27"/>
+      <c r="C219" s="27"/>
+      <c r="D219" s="27"/>
+      <c r="E219" s="27"/>
+      <c r="F219" s="27"/>
+      <c r="G219" s="27"/>
+      <c r="H219" s="28"/>
     </row>
     <row r="220" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A220" s="23" t="s">
+      <c r="A220" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="B220" s="24"/>
-      <c r="C220" s="24"/>
-      <c r="D220" s="25"/>
+      <c r="B220" s="22"/>
+      <c r="C220" s="22"/>
+      <c r="D220" s="23"/>
       <c r="E220" s="7"/>
       <c r="F220" s="7"/>
       <c r="G220" s="7"/>
@@ -7369,12 +7369,12 @@
       </c>
     </row>
     <row r="239" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A239" s="23" t="s">
+      <c r="A239" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B239" s="24"/>
-      <c r="C239" s="24"/>
-      <c r="D239" s="25"/>
+      <c r="B239" s="22"/>
+      <c r="C239" s="22"/>
+      <c r="D239" s="23"/>
       <c r="E239" s="13">
         <v>172480327</v>
       </c>
@@ -7383,12 +7383,12 @@
       <c r="H239" s="7"/>
     </row>
     <row r="240" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A240" s="23" t="s">
+      <c r="A240" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B240" s="24"/>
-      <c r="C240" s="24"/>
-      <c r="D240" s="25"/>
+      <c r="B240" s="22"/>
+      <c r="C240" s="22"/>
+      <c r="D240" s="23"/>
       <c r="E240" s="13">
         <v>172480327</v>
       </c>
@@ -7397,164 +7397,162 @@
       <c r="H240" s="7"/>
     </row>
     <row r="241" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A241" s="27" t="s">
+      <c r="A241" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="B241" s="27"/>
+      <c r="C241" s="27"/>
+      <c r="D241" s="27"/>
+      <c r="E241" s="27"/>
+      <c r="F241" s="27"/>
+      <c r="G241" s="27"/>
+      <c r="H241" s="28"/>
+    </row>
+    <row r="242" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A242" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="B242" s="27"/>
+      <c r="C242" s="27"/>
+      <c r="D242" s="27"/>
+      <c r="E242" s="27"/>
+      <c r="F242" s="27"/>
+      <c r="G242" s="27"/>
+      <c r="H242" s="28"/>
+    </row>
+    <row r="243" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A243" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B241" s="28"/>
-      <c r="C241" s="28"/>
-      <c r="D241" s="28"/>
-      <c r="E241" s="28"/>
-      <c r="F241" s="28"/>
-      <c r="G241" s="28"/>
-      <c r="H241" s="29"/>
-    </row>
-    <row r="242" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A242" s="23" t="s">
+      <c r="B243" s="27"/>
+      <c r="C243" s="27"/>
+      <c r="D243" s="27"/>
+      <c r="E243" s="27"/>
+      <c r="F243" s="27"/>
+      <c r="G243" s="27"/>
+      <c r="H243" s="28"/>
+    </row>
+    <row r="244" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A244" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="B242" s="24"/>
-      <c r="C242" s="24"/>
-      <c r="D242" s="25"/>
-      <c r="E242" s="7"/>
-      <c r="F242" s="7"/>
-      <c r="G242" s="7"/>
-      <c r="H242" s="7"/>
-    </row>
-    <row r="243" spans="1:8" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="A243" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B243" s="10">
+      <c r="B244" s="22"/>
+      <c r="C244" s="22"/>
+      <c r="D244" s="23"/>
+      <c r="E244" s="7"/>
+      <c r="F244" s="7"/>
+      <c r="G244" s="7"/>
+      <c r="H244" s="7"/>
+    </row>
+    <row r="245" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A245" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B245" s="10">
         <v>46141</v>
       </c>
-      <c r="C243" s="11" t="s">
+      <c r="C245" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="D243" s="9" t="s">
+      <c r="D245" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E243" s="12">
+      <c r="E245" s="12">
         <v>280600</v>
       </c>
-      <c r="F243" s="8"/>
-      <c r="G243" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H243" s="9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="244" spans="1:8" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="A244" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B244" s="10">
+      <c r="F245" s="8"/>
+      <c r="G245" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H245" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="246" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A246" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B246" s="10">
         <v>46141</v>
       </c>
-      <c r="C244" s="11" t="s">
+      <c r="C246" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="D244" s="9" t="s">
+      <c r="D246" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E244" s="12">
+      <c r="E246" s="12">
         <v>5617204</v>
       </c>
-      <c r="F244" s="8"/>
-      <c r="G244" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H244" s="9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="245" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A245" s="23" t="s">
+      <c r="F246" s="8"/>
+      <c r="G246" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H246" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="247" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A247" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B245" s="24"/>
-      <c r="C245" s="24"/>
-      <c r="D245" s="25"/>
-      <c r="E245" s="13">
+      <c r="B247" s="22"/>
+      <c r="C247" s="22"/>
+      <c r="D247" s="23"/>
+      <c r="E247" s="13">
         <v>5897804</v>
       </c>
-      <c r="F245" s="7"/>
-      <c r="G245" s="7"/>
-      <c r="H245" s="7"/>
-    </row>
-    <row r="246" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A246" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="B246" s="24"/>
-      <c r="C246" s="24"/>
-      <c r="D246" s="25"/>
-      <c r="E246" s="13">
-        <v>5897804</v>
-      </c>
-      <c r="F246" s="7"/>
-      <c r="G246" s="7"/>
-      <c r="H246" s="7"/>
-    </row>
-    <row r="247" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A247" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="B247" s="24"/>
-      <c r="C247" s="24"/>
-      <c r="D247" s="25"/>
-      <c r="E247" s="7"/>
       <c r="F247" s="7"/>
       <c r="G247" s="7"/>
       <c r="H247" s="7"/>
     </row>
     <row r="248" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A248" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="B248" s="24"/>
-      <c r="C248" s="24"/>
-      <c r="D248" s="25"/>
+      <c r="A248" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="B248" s="22"/>
+      <c r="C248" s="22"/>
+      <c r="D248" s="23"/>
       <c r="E248" s="13">
-        <v>178378131</v>
+        <v>5897804</v>
       </c>
       <c r="F248" s="7"/>
       <c r="G248" s="7"/>
       <c r="H248" s="7"/>
     </row>
     <row r="249" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A249" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="B249" s="24"/>
-      <c r="C249" s="24"/>
-      <c r="D249" s="25"/>
-      <c r="E249" s="13">
-        <v>178378131</v>
-      </c>
+      <c r="A249" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B249" s="22"/>
+      <c r="C249" s="22"/>
+      <c r="D249" s="23"/>
+      <c r="E249" s="7"/>
       <c r="F249" s="7"/>
       <c r="G249" s="7"/>
       <c r="H249" s="7"/>
     </row>
     <row r="250" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A250" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="B250" s="24"/>
-      <c r="C250" s="24"/>
-      <c r="D250" s="25"/>
-      <c r="E250" s="7"/>
+      <c r="A250" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B250" s="22"/>
+      <c r="C250" s="22"/>
+      <c r="D250" s="23"/>
+      <c r="E250" s="13">
+        <v>178378131</v>
+      </c>
       <c r="F250" s="7"/>
       <c r="G250" s="7"/>
       <c r="H250" s="7"/>
     </row>
     <row r="251" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A251" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="B251" s="24"/>
-      <c r="C251" s="24"/>
-      <c r="D251" s="25"/>
+      <c r="A251" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B251" s="22"/>
+      <c r="C251" s="22"/>
+      <c r="D251" s="23"/>
       <c r="E251" s="13">
         <v>178378131</v>
       </c>
@@ -7563,96 +7561,159 @@
       <c r="H251" s="7"/>
     </row>
     <row r="252" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A252" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="B252" s="24"/>
-      <c r="C252" s="24"/>
-      <c r="D252" s="25"/>
-      <c r="E252" s="13">
-        <v>178378131</v>
-      </c>
+      <c r="A252" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="B252" s="22"/>
+      <c r="C252" s="22"/>
+      <c r="D252" s="23"/>
+      <c r="E252" s="7"/>
       <c r="F252" s="7"/>
       <c r="G252" s="7"/>
       <c r="H252" s="7"/>
     </row>
     <row r="253" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A253" s="15"/>
+      <c r="A253" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B253" s="22"/>
+      <c r="C253" s="22"/>
+      <c r="D253" s="23"/>
+      <c r="E253" s="13">
+        <v>178378131</v>
+      </c>
+      <c r="F253" s="7"/>
+      <c r="G253" s="7"/>
+      <c r="H253" s="7"/>
     </row>
     <row r="254" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A254" s="15"/>
+      <c r="A254" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B254" s="22"/>
+      <c r="C254" s="22"/>
+      <c r="D254" s="23"/>
+      <c r="E254" s="13">
+        <v>178378131</v>
+      </c>
+      <c r="F254" s="7"/>
+      <c r="G254" s="7"/>
+      <c r="H254" s="7"/>
     </row>
     <row r="255" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A255" s="15"/>
     </row>
     <row r="256" spans="1:8" ht="11.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A256" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="B256" s="7"/>
-      <c r="C256" s="7"/>
-      <c r="D256" s="7"/>
-      <c r="E256" s="7"/>
+      <c r="A256" s="15"/>
     </row>
     <row r="257" spans="1:5" ht="11.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A257" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B257" s="13">
-        <v>1756914319</v>
-      </c>
-      <c r="C257" s="13">
-        <v>29678782</v>
-      </c>
-      <c r="D257" s="7"/>
-      <c r="E257" s="7"/>
+      <c r="A257" s="15"/>
     </row>
     <row r="258" spans="1:5" ht="11.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A258" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="B258" s="13">
-        <v>1727235537</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="B258" s="7"/>
       <c r="C258" s="7"/>
       <c r="D258" s="7"/>
       <c r="E258" s="7"/>
     </row>
-    <row r="261" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A261" s="26"/>
-      <c r="B261" s="26"/>
-      <c r="C261" s="17" t="s">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A259" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B259" s="13">
+        <v>1756914319</v>
+      </c>
+      <c r="C259" s="13">
+        <v>29678782</v>
+      </c>
+      <c r="D259" s="7"/>
+      <c r="E259" s="7"/>
+    </row>
+    <row r="260" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A260" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B260" s="13">
+        <v>1727235537</v>
+      </c>
+      <c r="C260" s="7"/>
+      <c r="D260" s="7"/>
+      <c r="E260" s="7"/>
+    </row>
+    <row r="261" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="262" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="263" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A263" s="33"/>
+      <c r="B263" s="33"/>
+      <c r="C263" s="17" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="262" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A262" s="4" t="s">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A264" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B262" s="1"/>
-      <c r="C262" s="4" t="s">
+      <c r="B264" s="1"/>
+      <c r="C264" s="4" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="263" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A263" s="18" t="s">
+    <row r="265" spans="1:5" ht="12.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A265" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="B263" s="6"/>
-      <c r="C263" s="18" t="s">
+      <c r="B265" s="6"/>
+      <c r="C265" s="18" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="265" spans="1:5" ht="12.15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A265" s="19" t="s">
+    <row r="267" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A267" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="B265" s="20" t="s">
+      <c r="B267" s="20" t="s">
         <v>143</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="49">
+  <mergeCells count="51">
+    <mergeCell ref="A242:H242"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A250:D250"/>
+    <mergeCell ref="A251:D251"/>
+    <mergeCell ref="A252:D252"/>
+    <mergeCell ref="A253:D253"/>
+    <mergeCell ref="A216:D216"/>
+    <mergeCell ref="A217:H217"/>
+    <mergeCell ref="A218:H218"/>
+    <mergeCell ref="A219:H219"/>
+    <mergeCell ref="A220:D220"/>
+    <mergeCell ref="A239:D239"/>
+    <mergeCell ref="A210:D210"/>
+    <mergeCell ref="A211:D211"/>
+    <mergeCell ref="A212:D212"/>
+    <mergeCell ref="A213:D213"/>
+    <mergeCell ref="A214:D214"/>
+    <mergeCell ref="A254:D254"/>
+    <mergeCell ref="A263:B263"/>
+    <mergeCell ref="A240:D240"/>
+    <mergeCell ref="A243:H243"/>
+    <mergeCell ref="A244:D244"/>
+    <mergeCell ref="A247:D247"/>
+    <mergeCell ref="A248:D248"/>
+    <mergeCell ref="A249:D249"/>
+    <mergeCell ref="A241:H241"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A215:D215"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A209:D209"/>
     <mergeCell ref="A48:D48"/>
     <mergeCell ref="H13:H14"/>
     <mergeCell ref="A15:H15"/>
@@ -7669,39 +7730,6 @@
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A44:D44"/>
     <mergeCell ref="A45:D45"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A215:D215"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="A50:H50"/>
-    <mergeCell ref="A51:H51"/>
-    <mergeCell ref="A52:H52"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A209:D209"/>
-    <mergeCell ref="A252:D252"/>
-    <mergeCell ref="A261:B261"/>
-    <mergeCell ref="A240:D240"/>
-    <mergeCell ref="A241:H241"/>
-    <mergeCell ref="A242:D242"/>
-    <mergeCell ref="A245:D245"/>
-    <mergeCell ref="A246:D246"/>
-    <mergeCell ref="A247:D247"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A248:D248"/>
-    <mergeCell ref="A249:D249"/>
-    <mergeCell ref="A250:D250"/>
-    <mergeCell ref="A251:D251"/>
-    <mergeCell ref="A216:D216"/>
-    <mergeCell ref="A217:H217"/>
-    <mergeCell ref="A218:H218"/>
-    <mergeCell ref="A219:H219"/>
-    <mergeCell ref="A220:D220"/>
-    <mergeCell ref="A239:D239"/>
-    <mergeCell ref="A210:D210"/>
-    <mergeCell ref="A211:D211"/>
-    <mergeCell ref="A212:D212"/>
-    <mergeCell ref="A213:D213"/>
-    <mergeCell ref="A214:D214"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cap nhat du lieu - 07/05/2026 15:20
</commit_message>
<xml_diff>
--- a/PM_092.xlsx
+++ b/PM_092.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TUAN HOC A.I\1. TCKT_PCVT\4. Công nghệ AI\KT SCL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{937510B4-8285-42FF-8E17-8B3A854FDBE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED5E2A54-56B2-46BF-96EE-032D3107D2EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{AC1AAD16-9061-42F9-B216-D7E5AB78D483}"/>
   </bookViews>
@@ -1770,6 +1770,19 @@
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1778,20 +1791,14 @@
     <xf numFmtId="0" fontId="21" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1805,13 +1812,6 @@
     <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2249,98 +2249,98 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="34" t="s">
+      <c r="A12" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="29" t="s">
+      <c r="A13" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="29" t="s">
+      <c r="D13" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="E13" s="31" t="s">
+      <c r="E13" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="F13" s="32"/>
-      <c r="G13" s="24" t="s">
+      <c r="F13" s="35"/>
+      <c r="G13" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="H13" s="30" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="30"/>
-      <c r="B14" s="30"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
+      <c r="A14" s="33"/>
+      <c r="B14" s="33"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="26" t="s">
+      <c r="A15" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="28"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="23"/>
     </row>
     <row r="16" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="28"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="23"/>
     </row>
     <row r="17" spans="1:8" ht="18.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="28"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="23"/>
     </row>
     <row r="18" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="23"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="28"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
@@ -2899,12 +2899,12 @@
       </c>
     </row>
     <row r="42" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="21" t="s">
+      <c r="A42" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="B42" s="22"/>
-      <c r="C42" s="22"/>
-      <c r="D42" s="23"/>
+      <c r="B42" s="27"/>
+      <c r="C42" s="27"/>
+      <c r="D42" s="28"/>
       <c r="E42" s="13">
         <v>103128028</v>
       </c>
@@ -2913,12 +2913,12 @@
       <c r="H42" s="7"/>
     </row>
     <row r="43" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="21" t="s">
+      <c r="A43" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B43" s="22"/>
-      <c r="C43" s="22"/>
-      <c r="D43" s="23"/>
+      <c r="B43" s="27"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="28"/>
       <c r="E43" s="13">
         <v>103128028</v>
       </c>
@@ -2927,24 +2927,24 @@
       <c r="H43" s="7"/>
     </row>
     <row r="44" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="21" t="s">
+      <c r="A44" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="B44" s="22"/>
-      <c r="C44" s="22"/>
-      <c r="D44" s="23"/>
+      <c r="B44" s="27"/>
+      <c r="C44" s="27"/>
+      <c r="D44" s="28"/>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
       <c r="H44" s="7"/>
     </row>
     <row r="45" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="21" t="s">
+      <c r="A45" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="B45" s="22"/>
-      <c r="C45" s="22"/>
-      <c r="D45" s="23"/>
+      <c r="B45" s="27"/>
+      <c r="C45" s="27"/>
+      <c r="D45" s="28"/>
       <c r="E45" s="13">
         <v>103128028</v>
       </c>
@@ -2953,12 +2953,12 @@
       <c r="H45" s="7"/>
     </row>
     <row r="46" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="21" t="s">
+      <c r="A46" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="B46" s="22"/>
-      <c r="C46" s="22"/>
-      <c r="D46" s="23"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="28"/>
       <c r="E46" s="13">
         <v>103128028</v>
       </c>
@@ -2967,24 +2967,24 @@
       <c r="H46" s="7"/>
     </row>
     <row r="47" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="21" t="s">
+      <c r="A47" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="B47" s="22"/>
-      <c r="C47" s="22"/>
-      <c r="D47" s="23"/>
+      <c r="B47" s="27"/>
+      <c r="C47" s="27"/>
+      <c r="D47" s="28"/>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
       <c r="G47" s="7"/>
       <c r="H47" s="7"/>
     </row>
     <row r="48" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="21" t="s">
+      <c r="A48" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="B48" s="22"/>
-      <c r="C48" s="22"/>
-      <c r="D48" s="23"/>
+      <c r="B48" s="27"/>
+      <c r="C48" s="27"/>
+      <c r="D48" s="28"/>
       <c r="E48" s="13">
         <v>103128028</v>
       </c>
@@ -2993,12 +2993,12 @@
       <c r="H48" s="7"/>
     </row>
     <row r="49" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="21" t="s">
+      <c r="A49" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="B49" s="22"/>
-      <c r="C49" s="22"/>
-      <c r="D49" s="23"/>
+      <c r="B49" s="27"/>
+      <c r="C49" s="27"/>
+      <c r="D49" s="28"/>
       <c r="E49" s="13">
         <v>103128028</v>
       </c>
@@ -3007,48 +3007,48 @@
       <c r="H49" s="7"/>
     </row>
     <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="26" t="s">
+      <c r="A50" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="B50" s="27"/>
-      <c r="C50" s="27"/>
-      <c r="D50" s="27"/>
-      <c r="E50" s="27"/>
-      <c r="F50" s="27"/>
-      <c r="G50" s="27"/>
-      <c r="H50" s="28"/>
+      <c r="B50" s="22"/>
+      <c r="C50" s="22"/>
+      <c r="D50" s="22"/>
+      <c r="E50" s="22"/>
+      <c r="F50" s="22"/>
+      <c r="G50" s="22"/>
+      <c r="H50" s="23"/>
     </row>
     <row r="51" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="26" t="s">
+      <c r="A51" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B51" s="27"/>
-      <c r="C51" s="27"/>
-      <c r="D51" s="27"/>
-      <c r="E51" s="27"/>
-      <c r="F51" s="27"/>
-      <c r="G51" s="27"/>
-      <c r="H51" s="28"/>
+      <c r="B51" s="22"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="22"/>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="22"/>
+      <c r="H51" s="23"/>
     </row>
     <row r="52" spans="1:8" ht="18.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="26" t="s">
+      <c r="A52" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B52" s="27"/>
-      <c r="C52" s="27"/>
-      <c r="D52" s="27"/>
-      <c r="E52" s="27"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="27"/>
-      <c r="H52" s="28"/>
+      <c r="B52" s="22"/>
+      <c r="C52" s="22"/>
+      <c r="D52" s="22"/>
+      <c r="E52" s="22"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="22"/>
+      <c r="H52" s="23"/>
     </row>
     <row r="53" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="21" t="s">
+      <c r="A53" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="B53" s="22"/>
-      <c r="C53" s="22"/>
-      <c r="D53" s="23"/>
+      <c r="B53" s="27"/>
+      <c r="C53" s="27"/>
+      <c r="D53" s="28"/>
       <c r="E53" s="7"/>
       <c r="F53" s="7"/>
       <c r="G53" s="7"/>
@@ -6775,12 +6775,12 @@
       </c>
     </row>
     <row r="209" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A209" s="21" t="s">
+      <c r="A209" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="B209" s="22"/>
-      <c r="C209" s="22"/>
-      <c r="D209" s="23"/>
+      <c r="B209" s="27"/>
+      <c r="C209" s="27"/>
+      <c r="D209" s="28"/>
       <c r="E209" s="13">
         <v>1475408160</v>
       </c>
@@ -6791,12 +6791,12 @@
       <c r="H209" s="7"/>
     </row>
     <row r="210" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A210" s="21" t="s">
+      <c r="A210" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B210" s="22"/>
-      <c r="C210" s="22"/>
-      <c r="D210" s="23"/>
+      <c r="B210" s="27"/>
+      <c r="C210" s="27"/>
+      <c r="D210" s="28"/>
       <c r="E210" s="13">
         <v>1445729378</v>
       </c>
@@ -6805,24 +6805,24 @@
       <c r="H210" s="7"/>
     </row>
     <row r="211" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A211" s="21" t="s">
+      <c r="A211" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="B211" s="22"/>
-      <c r="C211" s="22"/>
-      <c r="D211" s="23"/>
+      <c r="B211" s="27"/>
+      <c r="C211" s="27"/>
+      <c r="D211" s="28"/>
       <c r="E211" s="7"/>
       <c r="F211" s="7"/>
       <c r="G211" s="7"/>
       <c r="H211" s="7"/>
     </row>
     <row r="212" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A212" s="21" t="s">
+      <c r="A212" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="B212" s="22"/>
-      <c r="C212" s="22"/>
-      <c r="D212" s="23"/>
+      <c r="B212" s="27"/>
+      <c r="C212" s="27"/>
+      <c r="D212" s="28"/>
       <c r="E212" s="13">
         <v>1475408160</v>
       </c>
@@ -6833,12 +6833,12 @@
       <c r="H212" s="7"/>
     </row>
     <row r="213" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A213" s="21" t="s">
+      <c r="A213" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="B213" s="22"/>
-      <c r="C213" s="22"/>
-      <c r="D213" s="23"/>
+      <c r="B213" s="27"/>
+      <c r="C213" s="27"/>
+      <c r="D213" s="28"/>
       <c r="E213" s="13">
         <v>1445729378</v>
       </c>
@@ -6847,24 +6847,24 @@
       <c r="H213" s="7"/>
     </row>
     <row r="214" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A214" s="21" t="s">
+      <c r="A214" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="B214" s="22"/>
-      <c r="C214" s="22"/>
-      <c r="D214" s="23"/>
+      <c r="B214" s="27"/>
+      <c r="C214" s="27"/>
+      <c r="D214" s="28"/>
       <c r="E214" s="7"/>
       <c r="F214" s="7"/>
       <c r="G214" s="7"/>
       <c r="H214" s="7"/>
     </row>
     <row r="215" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A215" s="21" t="s">
+      <c r="A215" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="B215" s="22"/>
-      <c r="C215" s="22"/>
-      <c r="D215" s="23"/>
+      <c r="B215" s="27"/>
+      <c r="C215" s="27"/>
+      <c r="D215" s="28"/>
       <c r="E215" s="13">
         <v>1475408160</v>
       </c>
@@ -6875,12 +6875,12 @@
       <c r="H215" s="7"/>
     </row>
     <row r="216" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A216" s="21" t="s">
+      <c r="A216" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="B216" s="22"/>
-      <c r="C216" s="22"/>
-      <c r="D216" s="23"/>
+      <c r="B216" s="27"/>
+      <c r="C216" s="27"/>
+      <c r="D216" s="28"/>
       <c r="E216" s="13">
         <v>1445729378</v>
       </c>
@@ -6889,48 +6889,48 @@
       <c r="H216" s="7"/>
     </row>
     <row r="217" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A217" s="26" t="s">
+      <c r="A217" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="B217" s="27"/>
-      <c r="C217" s="27"/>
-      <c r="D217" s="27"/>
-      <c r="E217" s="27"/>
-      <c r="F217" s="27"/>
-      <c r="G217" s="27"/>
-      <c r="H217" s="28"/>
+      <c r="B217" s="22"/>
+      <c r="C217" s="22"/>
+      <c r="D217" s="22"/>
+      <c r="E217" s="22"/>
+      <c r="F217" s="22"/>
+      <c r="G217" s="22"/>
+      <c r="H217" s="23"/>
     </row>
     <row r="218" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A218" s="26" t="s">
+      <c r="A218" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B218" s="27"/>
-      <c r="C218" s="27"/>
-      <c r="D218" s="27"/>
-      <c r="E218" s="27"/>
-      <c r="F218" s="27"/>
-      <c r="G218" s="27"/>
-      <c r="H218" s="28"/>
+      <c r="B218" s="22"/>
+      <c r="C218" s="22"/>
+      <c r="D218" s="22"/>
+      <c r="E218" s="22"/>
+      <c r="F218" s="22"/>
+      <c r="G218" s="22"/>
+      <c r="H218" s="23"/>
     </row>
     <row r="219" spans="1:8" ht="18.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A219" s="26" t="s">
+      <c r="A219" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B219" s="27"/>
-      <c r="C219" s="27"/>
-      <c r="D219" s="27"/>
-      <c r="E219" s="27"/>
-      <c r="F219" s="27"/>
-      <c r="G219" s="27"/>
-      <c r="H219" s="28"/>
+      <c r="B219" s="22"/>
+      <c r="C219" s="22"/>
+      <c r="D219" s="22"/>
+      <c r="E219" s="22"/>
+      <c r="F219" s="22"/>
+      <c r="G219" s="22"/>
+      <c r="H219" s="23"/>
     </row>
     <row r="220" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A220" s="21" t="s">
+      <c r="A220" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="B220" s="22"/>
-      <c r="C220" s="22"/>
-      <c r="D220" s="23"/>
+      <c r="B220" s="27"/>
+      <c r="C220" s="27"/>
+      <c r="D220" s="28"/>
       <c r="E220" s="7"/>
       <c r="F220" s="7"/>
       <c r="G220" s="7"/>
@@ -7369,12 +7369,12 @@
       </c>
     </row>
     <row r="239" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A239" s="21" t="s">
+      <c r="A239" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="B239" s="22"/>
-      <c r="C239" s="22"/>
-      <c r="D239" s="23"/>
+      <c r="B239" s="27"/>
+      <c r="C239" s="27"/>
+      <c r="D239" s="28"/>
       <c r="E239" s="13">
         <v>172480327</v>
       </c>
@@ -7383,12 +7383,12 @@
       <c r="H239" s="7"/>
     </row>
     <row r="240" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A240" s="21" t="s">
+      <c r="A240" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B240" s="22"/>
-      <c r="C240" s="22"/>
-      <c r="D240" s="23"/>
+      <c r="B240" s="27"/>
+      <c r="C240" s="27"/>
+      <c r="D240" s="28"/>
       <c r="E240" s="13">
         <v>172480327</v>
       </c>
@@ -7397,48 +7397,48 @@
       <c r="H240" s="7"/>
     </row>
     <row r="241" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A241" s="26" t="s">
+      <c r="A241" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="B241" s="27"/>
-      <c r="C241" s="27"/>
-      <c r="D241" s="27"/>
-      <c r="E241" s="27"/>
-      <c r="F241" s="27"/>
-      <c r="G241" s="27"/>
-      <c r="H241" s="28"/>
+      <c r="B241" s="22"/>
+      <c r="C241" s="22"/>
+      <c r="D241" s="22"/>
+      <c r="E241" s="22"/>
+      <c r="F241" s="22"/>
+      <c r="G241" s="22"/>
+      <c r="H241" s="23"/>
     </row>
     <row r="242" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A242" s="26" t="s">
+      <c r="A242" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="B242" s="27"/>
-      <c r="C242" s="27"/>
-      <c r="D242" s="27"/>
-      <c r="E242" s="27"/>
-      <c r="F242" s="27"/>
-      <c r="G242" s="27"/>
-      <c r="H242" s="28"/>
+      <c r="B242" s="22"/>
+      <c r="C242" s="22"/>
+      <c r="D242" s="22"/>
+      <c r="E242" s="22"/>
+      <c r="F242" s="22"/>
+      <c r="G242" s="22"/>
+      <c r="H242" s="23"/>
     </row>
     <row r="243" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A243" s="26" t="s">
+      <c r="A243" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B243" s="27"/>
-      <c r="C243" s="27"/>
-      <c r="D243" s="27"/>
-      <c r="E243" s="27"/>
-      <c r="F243" s="27"/>
-      <c r="G243" s="27"/>
-      <c r="H243" s="28"/>
+      <c r="B243" s="22"/>
+      <c r="C243" s="22"/>
+      <c r="D243" s="22"/>
+      <c r="E243" s="22"/>
+      <c r="F243" s="22"/>
+      <c r="G243" s="22"/>
+      <c r="H243" s="23"/>
     </row>
     <row r="244" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A244" s="21" t="s">
+      <c r="A244" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="B244" s="22"/>
-      <c r="C244" s="22"/>
-      <c r="D244" s="23"/>
+      <c r="B244" s="27"/>
+      <c r="C244" s="27"/>
+      <c r="D244" s="28"/>
       <c r="E244" s="7"/>
       <c r="F244" s="7"/>
       <c r="G244" s="7"/>
@@ -7493,12 +7493,12 @@
       </c>
     </row>
     <row r="247" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A247" s="21" t="s">
+      <c r="A247" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="B247" s="22"/>
-      <c r="C247" s="22"/>
-      <c r="D247" s="23"/>
+      <c r="B247" s="27"/>
+      <c r="C247" s="27"/>
+      <c r="D247" s="28"/>
       <c r="E247" s="13">
         <v>5897804</v>
       </c>
@@ -7507,12 +7507,12 @@
       <c r="H247" s="7"/>
     </row>
     <row r="248" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A248" s="21" t="s">
+      <c r="A248" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B248" s="22"/>
-      <c r="C248" s="22"/>
-      <c r="D248" s="23"/>
+      <c r="B248" s="27"/>
+      <c r="C248" s="27"/>
+      <c r="D248" s="28"/>
       <c r="E248" s="13">
         <v>5897804</v>
       </c>
@@ -7521,24 +7521,24 @@
       <c r="H248" s="7"/>
     </row>
     <row r="249" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A249" s="21" t="s">
+      <c r="A249" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="B249" s="22"/>
-      <c r="C249" s="22"/>
-      <c r="D249" s="23"/>
+      <c r="B249" s="27"/>
+      <c r="C249" s="27"/>
+      <c r="D249" s="28"/>
       <c r="E249" s="7"/>
       <c r="F249" s="7"/>
       <c r="G249" s="7"/>
       <c r="H249" s="7"/>
     </row>
     <row r="250" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A250" s="21" t="s">
+      <c r="A250" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="B250" s="22"/>
-      <c r="C250" s="22"/>
-      <c r="D250" s="23"/>
+      <c r="B250" s="27"/>
+      <c r="C250" s="27"/>
+      <c r="D250" s="28"/>
       <c r="E250" s="13">
         <v>178378131</v>
       </c>
@@ -7547,12 +7547,12 @@
       <c r="H250" s="7"/>
     </row>
     <row r="251" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A251" s="21" t="s">
+      <c r="A251" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="B251" s="22"/>
-      <c r="C251" s="22"/>
-      <c r="D251" s="23"/>
+      <c r="B251" s="27"/>
+      <c r="C251" s="27"/>
+      <c r="D251" s="28"/>
       <c r="E251" s="13">
         <v>178378131</v>
       </c>
@@ -7561,24 +7561,24 @@
       <c r="H251" s="7"/>
     </row>
     <row r="252" spans="1:8" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A252" s="21" t="s">
+      <c r="A252" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="B252" s="22"/>
-      <c r="C252" s="22"/>
-      <c r="D252" s="23"/>
+      <c r="B252" s="27"/>
+      <c r="C252" s="27"/>
+      <c r="D252" s="28"/>
       <c r="E252" s="7"/>
       <c r="F252" s="7"/>
       <c r="G252" s="7"/>
       <c r="H252" s="7"/>
     </row>
     <row r="253" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A253" s="21" t="s">
+      <c r="A253" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="B253" s="22"/>
-      <c r="C253" s="22"/>
-      <c r="D253" s="23"/>
+      <c r="B253" s="27"/>
+      <c r="C253" s="27"/>
+      <c r="D253" s="28"/>
       <c r="E253" s="13">
         <v>178378131</v>
       </c>
@@ -7587,12 +7587,12 @@
       <c r="H253" s="7"/>
     </row>
     <row r="254" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A254" s="21" t="s">
+      <c r="A254" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="B254" s="22"/>
-      <c r="C254" s="22"/>
-      <c r="D254" s="23"/>
+      <c r="B254" s="27"/>
+      <c r="C254" s="27"/>
+      <c r="D254" s="28"/>
       <c r="E254" s="13">
         <v>178378131</v>
       </c>
@@ -7645,8 +7645,8 @@
     <row r="261" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="262" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="263" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A263" s="33"/>
-      <c r="B263" s="33"/>
+      <c r="A263" s="29"/>
+      <c r="B263" s="29"/>
       <c r="C263" s="17" t="s">
         <v>137</v>
       </c>
@@ -7679,38 +7679,9 @@
     </row>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="A242:H242"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A250:D250"/>
-    <mergeCell ref="A251:D251"/>
-    <mergeCell ref="A252:D252"/>
-    <mergeCell ref="A253:D253"/>
-    <mergeCell ref="A216:D216"/>
-    <mergeCell ref="A217:H217"/>
-    <mergeCell ref="A218:H218"/>
-    <mergeCell ref="A219:H219"/>
-    <mergeCell ref="A220:D220"/>
-    <mergeCell ref="A239:D239"/>
-    <mergeCell ref="A210:D210"/>
-    <mergeCell ref="A211:D211"/>
-    <mergeCell ref="A212:D212"/>
-    <mergeCell ref="A213:D213"/>
-    <mergeCell ref="A214:D214"/>
-    <mergeCell ref="A254:D254"/>
-    <mergeCell ref="A263:B263"/>
-    <mergeCell ref="A240:D240"/>
-    <mergeCell ref="A243:H243"/>
-    <mergeCell ref="A244:D244"/>
-    <mergeCell ref="A247:D247"/>
-    <mergeCell ref="A248:D248"/>
-    <mergeCell ref="A249:D249"/>
-    <mergeCell ref="A241:H241"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A215:D215"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="A50:H50"/>
-    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A45:D45"/>
     <mergeCell ref="A52:H52"/>
     <mergeCell ref="A53:D53"/>
     <mergeCell ref="A209:D209"/>
@@ -7727,9 +7698,38 @@
     <mergeCell ref="D13:D14"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="G13:G14"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A44:D44"/>
-    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A254:D254"/>
+    <mergeCell ref="A263:B263"/>
+    <mergeCell ref="A240:D240"/>
+    <mergeCell ref="A243:H243"/>
+    <mergeCell ref="A244:D244"/>
+    <mergeCell ref="A247:D247"/>
+    <mergeCell ref="A248:D248"/>
+    <mergeCell ref="A249:D249"/>
+    <mergeCell ref="A241:H241"/>
+    <mergeCell ref="A253:D253"/>
+    <mergeCell ref="A216:D216"/>
+    <mergeCell ref="A217:H217"/>
+    <mergeCell ref="A218:H218"/>
+    <mergeCell ref="A219:H219"/>
+    <mergeCell ref="A220:D220"/>
+    <mergeCell ref="A239:D239"/>
+    <mergeCell ref="A242:H242"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A250:D250"/>
+    <mergeCell ref="A251:D251"/>
+    <mergeCell ref="A252:D252"/>
+    <mergeCell ref="A210:D210"/>
+    <mergeCell ref="A211:D211"/>
+    <mergeCell ref="A212:D212"/>
+    <mergeCell ref="A213:D213"/>
+    <mergeCell ref="A214:D214"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A215:D215"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A51:H51"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>